<commit_message>
GiftLogs Sept 14 2024
</commit_message>
<xml_diff>
--- a/TestData/LV_T1508_T1511_T1514_VerifyTheRequiredFieldsValidationsAndHelpTextOfFields.xlsx
+++ b/TestData/LV_T1508_T1511_T1514_VerifyTheRequiredFieldsValidationsAndHelpTextOfFields.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AB81ED-5FE0-40AF-914E-678332FEC1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D5D2D4-7C6C-437B-8ACA-FE0833E8FE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -86,9 +86,6 @@
     <t>ContactName</t>
   </si>
   <si>
-    <t>Test External</t>
-  </si>
-  <si>
     <t>CongratulationsMsg</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>U.S. Dollar</t>
   </si>
   <si>
-    <t>Giorgia Cardia</t>
-  </si>
-  <si>
     <t>StandardTestCompany</t>
   </si>
   <si>
@@ -210,6 +204,12 @@
   </si>
   <si>
     <t>FVA</t>
+  </si>
+  <si>
+    <t>Olivia Ricketts</t>
+  </si>
+  <si>
+    <t>Giftlog Contact</t>
   </si>
 </sst>
 </file>
@@ -565,12 +565,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -589,12 +589,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -612,12 +612,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -633,12 +633,12 @@
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -648,7 +648,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>5</v>
@@ -657,7 +657,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>8</v>
@@ -675,7 +675,7 @@
         <v>1</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -683,7 +683,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
@@ -692,7 +692,7 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -701,16 +701,16 @@
         <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="J2" t="s">
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -724,53 +724,53 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -790,50 +790,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -841,7 +841,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -854,45 +854,45 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
         <v>50</v>
       </c>
-      <c r="C3" t="s">
-        <v>52</v>
-      </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
GiftLogs - Sept 17 24
</commit_message>
<xml_diff>
--- a/TestData/LV_T1508_T1511_T1514_VerifyTheRequiredFieldsValidationsAndHelpTextOfFields.xlsx
+++ b/TestData/LV_T1508_T1511_T1514_VerifyTheRequiredFieldsValidationsAndHelpTextOfFields.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D5D2D4-7C6C-437B-8ACA-FE0833E8FE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F356544C-ED05-47B5-B686-7B1F362CA0B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -206,10 +206,10 @@
     <t>FVA</t>
   </si>
   <si>
-    <t>Olivia Ricketts</t>
-  </si>
-  <si>
     <t>Giftlog Contact</t>
+  </si>
+  <si>
+    <t>Melissa Zatta</t>
   </si>
 </sst>
 </file>
@@ -560,7 +560,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -570,7 +570,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -631,7 +631,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -683,7 +683,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
@@ -704,7 +704,7 @@
         <v>20</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J2" t="s">
         <v>0</v>
@@ -854,7 +854,7 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -875,7 +875,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>47</v>

</xml_diff>